<commit_message>
Made changes in the code
</commit_message>
<xml_diff>
--- a/ExcelFiles/pdfData.xlsx
+++ b/ExcelFiles/pdfData.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG6"/>
+  <dimension ref="A1:AG20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1310,39 +1310,2005 @@
           <t>Public</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AA6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>83</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>www.thyrocare.com</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>['Thyroid testing', 'Over 920 tests', 'Her Check', 'Troponin I Heart Attack Risk Test', 'Jaanch', 'Aarogyam']</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>['Hospitals', 'Laboratories', 'Diagnostic centers', 'Nursing homes', 'Clinics', 'Doctors', 'Insurance partners']</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>['Navi Mumbai', 'Delhi', 'Bengaluru', 'Kolkata', 'Indore', 'Bengaluru', 'Mumbai', 'Mohali', 'Visakhapatnam', 'Goa', 'Kandivali', 'Amritsar', 'Bhopal', 'Chennai', 'Vizag', 'Hyderabad', 'Pune', 'Jaipur', 'Lucknow', 'Varanasi', 'Patna', 'Ranchi', 'New Delhi', 'Coimbatore', 'Kochi', 'Gujarat', 'Tanzania']</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EVEREST KANTO CYLINDER LTD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L29200MH1978PLC020434</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>204, Raheja Centre, Free Press Journal Marg, 214, Nariman Point, Mumbai - 400 021.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>204, Raheja Centre, Free Press Journal Marg, 214, Nariman Point, Mumbai - 400 021.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BSE, NSE</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2,244.15 Lakhs</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Suresh Surana &amp; Associates LLP</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>771.52 Crores</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>709.48 Crores</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>91 22 4926 8300 - 01</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>investors@ekc.in</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>1978</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>1222.9 Crores</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>392</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>294</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Clean Energy Solutions Company and a leading global manufacturer of seamless gas cylinders</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>www.everestkanto.com</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>['seamless steel cylinders', 'industrial cylinders', 'jumbo cylinders', 'composite cylinders', 'cascades', 'multiple element gas containers', 'specialized fire suppression and detection systems']</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>['City Gas Distribution Companies', 'CNG Vehicle Manufacturers']</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>['Tarapur (Maharashtra)', 'Kandla SEZ (Gujarat)', 'Jebel Ali Free Zone in Dubai', 'Pittsburgh (PA), USA']</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BIRLA PRECISION TECHNOLOGIES LTD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>L29220MH1986PLC041214</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>23, Birla Mansion No. 2, 1st Floor, D. D. Sathe Marg, Prarthana Samaj, Mumbai 400 004</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>23, Birla Mansion No. 2, 1st Floor, D. D. Sathe Marg, Prarthana Samaj, Mumbai, Maharashtra - 400 004</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>13,19,75,274</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>M /s. Valawat &amp; Associates Chartered Accountant</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>22,755.82 Lakhs</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>+91 022 - 23867498</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>info@birlaprecision.com</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>1937</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>22,755.82 Lakhs</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>747</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>industrial innovation, Cutting Tools, Tool Holders, and Automotive Precision Components</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>www.birlaprecision.com</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>['Cutting Tools', 'Tool Holders', 'Automotive Precision Components', 'AT3 class tool holders', 'advanced work holding solutions', 'versatile expanding mandrels', 'high-efficiency production boosters', 'cutting-edge capital equipment', 'precision boring bars', 'tailored tooling solutions', 'collet chucks', 'End mill adaptors', 'shell mill adaptors', 'work holdings', 'rotary coolant adaptors', 'right angle heads', 'multi-spindle heads', 'High-Speed Steel (HSS) cutting tools', 'high-precision carbide cutting tools', 'twist drills', 'reamers', 'taps', 'Birla Durotool', 'Engineering Files', 'Abrasive Cutting', 'Grinding', 'Polishing Disc', 'Hammer Drills', 'Masonry Drills', 'Wood Cutting/Marble Cutting saw blades', 'high-precision machined components', 'Spools', 'Fuel System Shafts', 'Rocker Levers', 'Bearing &amp; Turbine Housings', 'various Sub-Assemblies']</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>['OEMs']</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>['Mumbai', 'Nashik', 'Aurangabad', 'Chalisgaon']</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BAJAJ STEEL INDUSTRIES LTD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>L27100MH1961PLC011936</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>C - 108 , MIDC Industrial Area , Hingna , Nagpur – 440 016 (M.S.) INDIA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>C - 108 , MIDC Industrial Area , Hingna , Nagpur – 440 016</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BSE Limited</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>260.00</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>B. Chhawchharia &amp; Co., Chartered Accountants, Nagpur</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>50,837.28 lakhs</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>29,266.57 lakhs</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>07104-238101-20</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>cs_legal@bajajngp.com</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1961</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Ginning Machinery, Cotton Ginning, Cotton Cleaning, Cotton Conveying, Cotton Humidification System, Cotton Baling Presses, Saw Ginning, Double Roller Ginning, Rotary Knife Rotobar Ginning, Single Roller Ginning, delinting &amp; decorticating machinery, automation etc.</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://bajajngp.com/investor-relations/annual-report/</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>['BAJAJ COTTON GINNING MACHINERY', 'BAJAJ DOUBLE ROLLER GIN WITH AUTO FEEDER', 'BAJAJ SINGLE ROLLER GIN WITH AUTO FEEDER', 'BAJAJ CONTINENTAL ROTO BAR GIN WITH FEEDER', 'BAJAJ CONTINENTAL SAW GIN WITH FEEDER', 'Pre-Engineered Steel Buildings', 'Electrical Panels, and other Electronic Equipments’', 'General and Heavy Engineering Parts etc.', 'Passenger Boarding Bridge', 'Duct System, Conveyors, Steel Doors, Suction Fans &amp; Blowers, Fire Fighting and Hydrant Systems']</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>['C - 54 , Hingna MIDC , Nagpur – 440 016 (M.S.) INDIA', 'Plot No. C - 22 , MIDC , Hingna , Industrial Area , Nagpur – 440 016 (M.S.) INDIA', 'Plot No. G - 108 , Butibori MIDC , Nagpur (M.S.) , - 441 108 INDIA', 'Plot No. K 63 , Butibori MIDC , Nagpur (M.S.) , - 441 108 INDIA', 'G - 6 &amp; G - 7 , MIDC , Hingna , Nagpur - 440 016 (M.S.) INDIA', 'G - 10 , MIDC , Hingna , Nagpur – 440 016 (M.S.) INDIA', 'Plot No. XI - 73 , MIDC , Hingna , Nagpur – 440 016 (M.S.) INDIA', 'Plot No. XI - 75 , Hingna MIDC , Nagpur – 440 016 (M.S.) INDIA', 'D - 4 , MIDC , Hingna , Nagpur – 440 016 (M.S.) INDIA', 'D - 5/2 , MIDC , Hingna , Nagpur – 440 016 (M.S.) INDIA']</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Affordable Robotic &amp; Automation Ltd</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>L29299PN2010PLC135298</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Village Wadki, Gat No. 1209, Tal Haveli, Dist. Pune – 412308 Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Gat No 1209, Village Wadaki, Tal Haveli, Pune - Saswad Road, Pune 412308, Maharashtra, India.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>BSE SME platform</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>11,24,62,660</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>16309.93 Lakhs</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>7720018914</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>cs@arapl.co.in</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Manohar Padole and Milind Padole</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>January 12, 2010</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>16340.41</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>350+</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Robotics &amp; Automation</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>www.arapl.co.in</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>['Industrial Automation', 'Multi-level Car Parking']</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>['Pune, Maharashtra']</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SHANTHI GEARS LTD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L29130TZ1972PLC000649</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>304-A, Trichy Road, Singanallur, Coimbatore - 641 005</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>304-A, Trichy Road, Singanallur, Coimbatore - 641 005</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>₹ 7.67 Cr</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>₹ 536.05 Crores</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>₹ 345.31 Crores</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>+91 422 4545745</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>info@shanthigears.murugappa.com</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>₹ 536.05 Crores</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>1159</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>386</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Industrial Gear</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="AC11" t="n">
+        <v>55</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>www.shanthigears.com</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>['Gears', 'Gearboxes', 'Geared Motors', 'Gear Assemblies']</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>['OEMs', 'dealers', 'end users', 'mineral processing', 'mining', 'off-highway vehicles', 'rubber &amp; plastics', 'extruders', 'power generation', 'wind energy', 'general engineering', 'steel', 'textiles', 'railways', 'chemical', 'fertilizers', 'non-ferrous metals', 'pumps', 'valves', 'blowers', 'compressors', 'lifts', 'conveyors', 'cranes', 'material handling', 'pulp &amp; paper', 'cement', 'sugar', 'foundry', 'conveyor systems', 'aviation', 'defense', 'textile mills', 'food processing']</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>['C Unit, Avinashi Road, Muthugoundenpudur, Coimbatore', 'D Unit, K. Krishnapuram, Tirupur', 'F Unit, Kannampalayam, Coimbatore']</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PENNAR INDUSTRIES LTD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L27109TG1975PLC001919</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2-91/14/8/PIL/10 &amp; 11, 7th Floor, Whitefields, Kondapur, Serilingampally, Hyderabad, K.V. Rangareddy - 500084</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2-91/14/8/PIL/10 &amp; 11, 7th Floor, Whitefields, Kondapur, Serilingampally, Hyderabad, K.V. Rangareddy - 500084</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>67,47,31,155 INR</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>3,13,057 Lakhs</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>78.817 Crores</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>+91 40 41923108</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>corporatecommunications@pennarindia.com</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Nrupender Rao</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Chairman Emeritus</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>3,130.57 Crores</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>4,800+</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>2,207</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC12" t="n">
+        <v>135</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https:// www.pennarindia.com/ index.php</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>['Structural railway components for Coaches, Wagons, and other parts', 'Industrial components to Automobile &amp; White Goods sectors', 'Precision Tubes', 'ESP electrodes, building materials, special grade CRSS, and solar MMS']</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>['Integral Coach Factory', 'Texmaco Rail &amp; Engineering Limited', 'Wabtec India Industrial (P) Limited', 'Controller of Stores (Mcf)', 'RITES Limited']</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>['IDA Patancheru, Medak (Dist.), Telangana', 'Isnapur Village, Medak (Dist.), Telangana', 'Survey 24, 27 to 38, Velchal (V) Mominpet, Vikarabad District, Telangana', 'Kannikaipair Village, Uthukottai Tq Thiruvallur Dist., Tamil Nadu', 'J-72, MIDC, Tarapur, Maharashtra', 'Chandapur Village, Sadasivpet Mandal, Medak (Dist.)', '186/A &amp; 188/A, IDA Mallapur, RR (Dist.)', '49/23, 49/10, 49/3, 49/2, 49/5, 49/7, 50/19, 50/5, 50/11, 50, Pudhukudi Thenpati, Pudukudi, Thanjavur (Dt), Tamil Nadu', 'Khata No. 00079, Plot No. 200, Rampur Nihastha, Lalgunj Tehsil, Raebareli District, Uttar Pradesh', '214 Fountainhead Road Portland TN 37148 USA']</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SHIVALIK BIMETAL CONTROLS LTD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>L27101HP1984PLC005862</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>16-18, New Electronics Complex, Chambaghat, Distt. Solan - 173213, Himachal Pradesh.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>H-2, Suneja Chambers, 2nd Floor, Alaknanda Commercial Complex, New Delhi - 110019.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>11,52,08,400</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>44,940.44</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>342 Crore</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>+91-1792-230578</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>investor@shivalikbimetals.com</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>449.40 Crore</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>875</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Process and Product Engineering</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>47 days</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>www.shivalikbimetals.com</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>['Thermostatic Bimetal / Trimetal strips', 'Components', 'EB welded products with multi gauge', 'Cold Bonded Bimetal Strips and Parts', 'Shunt resistors', 'Silver &amp; electrical contacts']</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>['Original Equipment Manufacturers (OEMs)']</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>['Plot No. 16-18, New Electronic Complex, Chambaghat', 'Mauja Basal Patti, Kather']</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Welspun Specialty Solutions Ltd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>L27100GJ1980PLC020358</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Plot No. 1, G. I. D. C. Industrial Estate, Valia Road, Jhagadia, Dist. Bharuch, Gujarat 393 110</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>5th Floor, Welspun House, Kamala Mills Compound, S. B. Marg, Lower Parel (W), Mumbai 400 013</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Rs. 368,95,77,646/-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>JMJ &amp; Associates LLP</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Secretarial Audit</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Rs. 718.2 crores</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Rs. 111.31 crores</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>022 6133 6796 / 2490 8000</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>companysecretary_wssl@welspun.com</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1980</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Rs. 71,817 Lakhs</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>760</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Alloy &amp; Stainless Steel Bars &amp; Tubes</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AB14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>www.thyrocare.com</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>['Thyroid testing', 'Over 920 tests', 'Her Check', 'Troponin I Heart Attack Risk Test', 'Jaanch', 'Aarogyam']</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>['Hospitals', 'Laboratories', 'Diagnostic centers', 'Nursing homes', 'Clinics', 'Doctors', 'Insurance partners']</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>['Navi Mumbai', 'Delhi', 'Bengaluru', 'Kolkata', 'Indore', 'Bengaluru', 'Mumbai', 'Mohali', 'Visakhapatnam', 'Goa', 'Kandivali', 'Amritsar', 'Bhopal', 'Chennai', 'Vizag', 'Hyderabad', 'Pune', 'Jaipur', 'Lucknow', 'Varanasi', 'Patna', 'Ranchi', 'New Delhi', 'Coimbatore', 'Kochi', 'Gujarat', 'Tanzania']</t>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>www.welspunspecialty.com</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>['Billets', 'Ingots', 'Black Bars', 'Tubes', 'Pipes', 'Hollow Profiles', 'Tube or Pipe Fittings']</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>['Jhagadia, Dist. Bharuch, Gujarat']</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KALYANI STEELS LTD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>L27104MH1973PLC016350</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mundhwa, Pune – 411 036, India</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Corporate Building, 2nd Floor, Mundhwa, Pune – 411 036, India</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>218.64 Million</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Care Ratings Limited</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>CARE AA Stable (Double A; Outlook: Stable) CARE A1+ (A One Plus) CARE A1+ (A One Plus)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>19,594.92 Million</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>16,914.44 Million</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>+91 20 6621 5000</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>investor@kalyanisteels.com</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>B. N. Kalyani</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Chairman</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>19,594.92 Million</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Forging and Engineering quality carbon and alloy steels</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>65.53</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>www.kalyanisteels.com</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>['Rolled Products', 'As Cast Blooms &amp; Rounds', 'Pig Iron', 'Foundry Coke']</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>['Bharat Forge Limited', 'Kalyani Technoforge Limited and its subsidiary']</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>['Ginigeri, Taluk and District Koppal, Karnataka']</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ELECTROTHERM (INDIA) LTD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>L29249GJ1986PLC009126</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>A - 1 , Skylark Apartment , Satellite Road , Satellite , Ahmedabad - 380 015.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Survey No. 72 , Palodia , ( Via Thaltej , Ahmedabad ) , Gujarat - 382 115 , India.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>4275.84</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>(722.22)</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>+ 91 - 79 - 2676 8844</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>sec@electrotherm.com</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>4275.84</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>2431</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Technologies</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>www.electrotherm.com</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>['Induction Furnaces', 'TMT Bars', 'Ductile Iron Pipes', 'Electric Vehicles', 'Transformers']</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>['Angul', 'Bangalore', 'Bangladesh', 'Bellary', 'Chennai', 'Coimbatore', 'Delhi', 'Ghaziabad', 'Goa', 'Hyderabad', 'Jaipur', 'Jalna', 'Jalandhar', 'Jamnagar', 'Jamshdepur', 'Kanpur', 'Koderma', 'Kolhapur', 'Kolkata', 'Ludhiana', 'Mandi Gobindgarh', 'Mumbai', 'Nagpur', 'Nasik', 'Panaji', 'Pune', 'Raipur', 'Raigarh', 'Rajkot', 'Rourkela', 'Sambalpur']</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ratnaveer Precision Engineering Ltd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>L27108GJ2002PLC040488</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>E - 77, GIDC Savli ( Manjusar ) Dist. Vadodara Gujarat - 391 776</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>703/704, “ OCEAN ”, Vikram Sarabhai Campus, Vadi Wadi, Vadodara, Gujarat 390 023</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>NSE-BSE</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>48,49,90,400</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>M / s . Pankaj R Shah &amp; Associates Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>6024.00</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2,521.14</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>8487878075</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>cs@ratnaveer.com</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Vijay R Sanghvi</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>20.02.2002</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>6024.00</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Precision engineering sector, specializing in the manufacture of high-quality stainless steel products</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>www.ratnaveer.com</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>['stainless steel finishing sheets', 'washers', 'solar roofing hooks', 'pipes and tubes']</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>['Vadodara, Gujarat', 'Unit - IV : Vatva, Ahmedabad', 'Unit - III : Waghodia, Vadodara', 'Unit - I and Unit - II : GIDC, Savli, Vadodara']</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>UNI ABEX ALLOY PRODUCTS LTD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>L27100MH1972PLC015950</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Liberty Building, Sir Vithaldas Thackersey Marg, Mumbai - 400 020,</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Phir oze Jeejebhoy Towers, Dalal Street, Fort, Mumbai - 400 001</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>197.50 lakhs</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Walker Chandiok &amp; Company LLP</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>17,999 lakhs</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>11,318</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>+91-22-22084436</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>companysecretary@uniabex.com</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>17,999 lakhs</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Metallurgical</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>www.uniabex.com</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>['centrifugal and static castings', 'heat, wear and corrosion-resistant stainless-steel alloys', 'alloy steel castings', 'reformer tubes', 'assemblies', 'radiant tubes', 'retort tubes', 'air injection tubes', 'tube support castings', 'tube sheets', 'header assemblies']</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>['marquee brands across various industry segments', 'refineries', 'petrochemicals', 'fertilizers', 'separators/decanter', 'iron and steel']</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>['Dharwad, Karnataka - 580 011, India']</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tiger Logistics (India) Ltd</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>L74899DL2000PLC105817</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>D-174, GF, Okhla Industrial Area, Phase-1, New Delhi - 110020 (India)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>804A-807, 8th Floor, Skylark Building 60, Nehru Place, New Delhi - 110019, India</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>10,57,25,000</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>24,025.85 Lacs</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>100 Cr</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>011-4735 1111</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>csvishal@tigerlogistics.in</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>24,025.85 Lacs</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>www.tigerlogistics.in</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>['International Cargo', 'Project Logistics', 'Defense Logistics', 'Cold Chain Logistics', 'Freight Jar']</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>['HPCL', 'BHEL']</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>['New Delhi (HQ)', 'Mumbai', 'Ahmedabad', 'Chennai', 'Gandhidham', 'Bengaluru', 'Nashik', 'Mundra', 'Nhava Sheva', 'Chennai ICD', 'Dadri ICD', 'Kathuwas ICD', 'Tughlakabad ICD', 'Garhi ICD']</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Uni Abex Ltd</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Industrial Products</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>L27100MH1972PLC015950</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Liberty Building, Sir Vithaldas Thackersey Marg, Mumbai - 400 020,</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Phir oze Jeejebhoy Towers, Dalal Street, Fort, Mumbai - 400 001</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>197.50 lakhs</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Walker Chandiok &amp; Company LLP</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Statutory Auditors</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>17,999 lakhs</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>11,318</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>+91-22-22084436</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>companysecretary@uniabex.com</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>17,998.69</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Metallurgical</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>www.uniabex.com</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>['centrifugal and static castings', 'heat, wear and corrosion-resistant stainless-steel alloys', 'alloy steel castings', 'reformer tubes and assemblies', 'bimetallic run out transport rolls', 'air injection tubes', '50 chrome - 50 Nickel Niobium alloy components', 'duplex stainless-steel alloy components', 'reformer tubes', 'bronze alloy castings', 'Hastelloy assemblies', 'diffuser casting', '17-4 PH &amp; Stellite alloys', 'centrifugally cast pipe supports', 'cold-cast beams', 'UM-Co grade parts']</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>['marquee brands across various industry segments', 'refineries', 'petrochemicals', 'fertilizers', 'separators/decanter', 'iron and steel', 'Indian Navy', 'Tata Group', 'OEM in Europe', 'US based global manufacturer']</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>['Mumbai, Maharashtra', 'Dharwad, Karnataka']</t>
         </is>
       </c>
     </row>

</xml_diff>